<commit_message>
switched back to analysis tab
</commit_message>
<xml_diff>
--- a/output3.xlsx
+++ b/output3.xlsx
@@ -1732,7 +1732,7 @@
         <v>-4.461376877758858</v>
       </c>
       <c r="J40" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="41">
@@ -3364,7 +3364,7 @@
         <v>-4.430787850675006</v>
       </c>
       <c r="J91" t="n">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="92">
@@ -5542,7 +5542,7 @@
         <v>-4.40502661773105</v>
       </c>
       <c r="J40" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="41">
@@ -7174,7 +7174,7 @@
         <v>-4.403587686935824</v>
       </c>
       <c r="J91" t="n">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="92">
@@ -9352,7 +9352,7 @@
         <v>-4.538007065084413</v>
       </c>
       <c r="J40" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="41">
@@ -10984,7 +10984,7 @@
         <v>-4.512180816993867</v>
       </c>
       <c r="J91" t="n">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="92">
@@ -13162,7 +13162,7 @@
         <v>-4.512110319708396</v>
       </c>
       <c r="J40" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="41">
@@ -14794,7 +14794,7 @@
         <v>-4.350965460417323</v>
       </c>
       <c r="J91" t="n">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="92">

</xml_diff>